<commit_message>
add everything going dominicano
</commit_message>
<xml_diff>
--- a/crypto_book.xlsx
+++ b/crypto_book.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jacob\bolt-hub\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB591C49-12D0-4379-BCA6-2DFE8D451CC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{360D8B1D-9A40-42E8-ABA4-EB6264C1C0B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-33765" yWindow="-21720" windowWidth="51840" windowHeight="21120" xr2:uid="{A613C9E8-9111-426C-AD0D-0425AFDE0B97}"/>
   </bookViews>
@@ -247,27 +247,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/volatileDependencies.xml><?xml version="1.0" encoding="utf-8"?>
-<volTypes xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <volType type="realTimeData">
-    <main first="pyxll.rtd">
-      <tp t="e">
-        <v>#N/A</v>
-        <stp/>
-        <stp>{CE91D9F9-C8CB-43A5-AE1B-3541C17B1734}</stp>
-        <tr r="C2" s="1"/>
-      </tp>
-      <tp t="e">
-        <v>#N/A</v>
-        <stp/>
-        <stp>{CD617962-CDD2-4F8C-9659-F6B58E16EF8F}</stp>
-        <tr r="B2" s="1"/>
-      </tp>
-    </main>
-  </volType>
-</volTypes>
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -436,79 +415,79 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="25"/>
                 <c:pt idx="0">
-                  <c:v>0.74986119611660285</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.7213035754450916</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.69507449686154033</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.67117396036594934</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.64960196595831832</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.63035851363864748</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.61344360340693671</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.59885723526318602</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.58659940920739539</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.57667012523956485</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.56906938335969448</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.56379718356778419</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.56085352586383386</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.56023841024784382</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.56195183671981375</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.56599380527974386</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.57236431592763393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.58106336866348418</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.59209096348729451</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.60544710039906491</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.62113177939879549</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.63914500048648615</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.65948676366213677</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.68215706892574757</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.70715591627731855</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1661,17 +1640,17 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" cm="1">
-        <f t="array" ref="B2">_xll.get_stock_price_ticking(B1)</f>
-        <v>1649.72998046875</v>
-      </c>
-      <c r="C2" s="1" cm="1">
-        <f t="array" ref="C2">_xll.get_stock_price_ticking(C1)</f>
-        <v>85454.734375</v>
+      <c r="B2" s="1" t="e" cm="1">
+        <f t="array" aca="1" ref="B2" ca="1">_xll.get_stock_price_ticking(B1)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C2" s="1" t="e" cm="1">
+        <f t="array" aca="1" ref="C2" ca="1">_xll.get_stock_price_ticking(C1)</f>
+        <v>#VALUE!</v>
       </c>
       <c r="D2" s="1"/>
       <c r="X2" t="str" cm="1">
-        <f t="array" ref="X2:AE21">_xll.get_positions()</f>
+        <f t="array" ref="X2:AE22">_xll.get_positions()</f>
         <v>ticker</v>
       </c>
       <c r="Y2" t="str">
@@ -1772,11 +1751,11 @@
       </c>
       <c r="B5" s="2">
         <f ca="1">NOW()</f>
-        <v>45759.96848333333</v>
+        <v>45760.082087037037</v>
       </c>
       <c r="C5" s="2">
         <f ca="1">NOW()</f>
-        <v>45759.96848275463</v>
+        <v>45760.082087037037</v>
       </c>
       <c r="X5" t="str">
         <v>KXBTCMAXY-25-DEC31-499999.99</v>
@@ -1809,11 +1788,11 @@
       </c>
       <c r="B6">
         <f ca="1">($E$1-B5)/365</f>
-        <v>0.71789456621005376</v>
+        <v>0.71758332318619966</v>
       </c>
       <c r="C6">
         <f ca="1">($E$1-C5)/365</f>
-        <v>0.71789456779553473</v>
+        <v>0.71758332318619966</v>
       </c>
       <c r="Q6" t="str" cm="1">
         <f t="array" ref="Q6">_xll.get_cwd()</f>
@@ -1847,83 +1826,83 @@
     <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="Q7" cm="1">
         <f t="array" ref="Q7">_xll.get_balance()</f>
-        <v>633.13</v>
+        <v>632.75</v>
       </c>
       <c r="X7" t="str">
-        <v>KXBTCMAXY-25-DEC31-179999.99</v>
+        <v>KXBTCMAXY-25-DEC31-124999.99</v>
       </c>
       <c r="Y7">
-        <v>238013</v>
+        <v>679762</v>
       </c>
       <c r="Z7">
-        <v>543</v>
+        <v>1</v>
       </c>
       <c r="AA7">
-        <v>7034</v>
+        <v>36</v>
       </c>
       <c r="AB7">
-        <v>-3478</v>
+        <v>25474</v>
       </c>
       <c r="AC7">
-        <v>543</v>
+        <v>1000</v>
       </c>
       <c r="AD7">
-        <v>504</v>
+        <v>3640</v>
       </c>
       <c r="AE7" t="str">
-        <v>2025-04-07T02:14:02.61871Z</v>
+        <v>2025-04-12T22:04:01.23325Z</v>
       </c>
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="X8" t="str">
-        <v>KXBTCMAXY-25-DEC31-299999.99</v>
+        <v>KXBTCMAXY-25-DEC31-179999.99</v>
       </c>
       <c r="Y8">
-        <v>564223</v>
+        <v>238013</v>
       </c>
       <c r="Z8">
-        <v>-5780</v>
+        <v>543</v>
       </c>
       <c r="AA8">
-        <v>548509</v>
+        <v>7034</v>
       </c>
       <c r="AB8">
-        <v>186</v>
+        <v>-3478</v>
       </c>
       <c r="AC8">
-        <v>3445</v>
+        <v>543</v>
       </c>
       <c r="AD8">
-        <v>1128</v>
+        <v>504</v>
       </c>
       <c r="AE8" t="str">
-        <v>2025-04-12T17:57:55.053573Z</v>
+        <v>2025-04-07T02:14:02.61871Z</v>
       </c>
     </row>
     <row r="9" spans="1:31" x14ac:dyDescent="0.25">
       <c r="X9" t="str">
-        <v>KXBTCMAXY-25-DEC31-249999.99</v>
+        <v>KXBTCMAXY-25-DEC31-299999.99</v>
       </c>
       <c r="Y9">
-        <v>873424</v>
+        <v>564223</v>
       </c>
       <c r="Z9">
-        <v>-4539</v>
+        <v>-5780</v>
       </c>
       <c r="AA9">
-        <v>420988</v>
+        <v>548509</v>
       </c>
       <c r="AB9">
-        <v>17664</v>
+        <v>186</v>
       </c>
       <c r="AC9">
-        <v>4500</v>
+        <v>3445</v>
       </c>
       <c r="AD9">
-        <v>2582</v>
+        <v>1128</v>
       </c>
       <c r="AE9" t="str">
-        <v>2025-04-09T01:05:01.757685Z</v>
+        <v>2025-04-12T17:57:55.053573Z</v>
       </c>
     </row>
     <row r="10" spans="1:31" x14ac:dyDescent="0.25">
@@ -1934,28 +1913,28 @@
         <v>14</v>
       </c>
       <c r="X10" t="str">
-        <v>KXGREENLAND-29</v>
+        <v>KXBTCMAXY-25-DEC31-249999.99</v>
       </c>
       <c r="Y10">
-        <v>913201</v>
+        <v>873424</v>
       </c>
       <c r="Z10">
-        <v>-1955</v>
+        <v>-4539</v>
       </c>
       <c r="AA10">
-        <v>141219</v>
+        <v>420988</v>
       </c>
       <c r="AB10">
-        <v>-4881</v>
+        <v>17664</v>
       </c>
       <c r="AC10">
-        <v>1841</v>
+        <v>4500</v>
       </c>
       <c r="AD10">
-        <v>1331</v>
+        <v>2582</v>
       </c>
       <c r="AE10" t="str">
-        <v>2025-04-12T13:36:11.493404Z</v>
+        <v>2025-04-09T01:05:01.757685Z</v>
       </c>
     </row>
     <row r="11" spans="1:31" x14ac:dyDescent="0.25">
@@ -2009,28 +1988,28 @@
         <v>23</v>
       </c>
       <c r="X11" t="str">
-        <v>KXH1B-29</v>
+        <v>KXGREENLAND-29</v>
       </c>
       <c r="Y11">
-        <v>323266</v>
+        <v>913201</v>
       </c>
       <c r="Z11">
-        <v>-234</v>
+        <v>-1955</v>
       </c>
       <c r="AA11">
-        <v>11325</v>
+        <v>141219</v>
       </c>
       <c r="AB11">
-        <v>5559</v>
+        <v>-4881</v>
       </c>
       <c r="AC11">
-        <v>215</v>
+        <v>1841</v>
       </c>
       <c r="AD11">
-        <v>0</v>
+        <v>1331</v>
       </c>
       <c r="AE11" t="str">
-        <v>2025-04-12T05:46:31.43372Z</v>
+        <v>2025-04-12T13:36:11.493404Z</v>
       </c>
     </row>
     <row r="12" spans="1:31" x14ac:dyDescent="0.25">
@@ -2053,7 +2032,7 @@
         <v>50</v>
       </c>
       <c r="G12">
-        <v>930</v>
+        <v>1353</v>
       </c>
       <c r="H12" t="str">
         <v>less</v>
@@ -2064,37 +2043,37 @@
       <c r="J12">
         <v>1</v>
       </c>
-      <c r="K12" cm="1">
+      <c r="K12" t="e" cm="1">
         <f t="array" aca="1" ref="K12" ca="1">_xll.price_one_touch($C$2,I12,J12,$C$3,$C$6)</f>
-        <v>0.82041282221946887</v>
-      </c>
-      <c r="M12" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M12" t="e" cm="1">
         <f t="array" aca="1" ref="M12" ca="1">_xll.one_touch_delta($C$2,I12,J12,$C$3,$C$6)</f>
-        <v>-8.1978471831882782E-3</v>
+        <v>#VALUE!</v>
       </c>
       <c r="X12" t="str">
-        <v>KXCANADAPM-45-L</v>
+        <v>KXH1B-29</v>
       </c>
       <c r="Y12">
-        <v>3479711</v>
+        <v>323266</v>
       </c>
       <c r="Z12">
-        <v>-7000</v>
+        <v>-234</v>
       </c>
       <c r="AA12">
-        <v>251557</v>
+        <v>11325</v>
       </c>
       <c r="AB12">
-        <v>-205253</v>
+        <v>5559</v>
       </c>
       <c r="AC12">
-        <v>4000</v>
+        <v>215</v>
       </c>
       <c r="AD12">
-        <v>12724</v>
+        <v>0</v>
       </c>
       <c r="AE12" t="str">
-        <v>2025-04-10T12:09:54.480709Z</v>
+        <v>2025-04-12T05:46:31.43372Z</v>
       </c>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.25">
@@ -2111,13 +2090,13 @@
         <v>33</v>
       </c>
       <c r="E13">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F13">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G13">
-        <v>604</v>
+        <v>560</v>
       </c>
       <c r="H13" t="str">
         <v>less</v>
@@ -2128,37 +2107,37 @@
       <c r="J13">
         <v>1</v>
       </c>
-      <c r="K13" cm="1">
+      <c r="K13" t="e" cm="1">
         <f t="array" aca="1" ref="K13" ca="1">_xll.price_one_touch($C$2,I13,J13,$C$3,$C$6)</f>
-        <v>0.69183983239896607</v>
-      </c>
-      <c r="M13" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M13" t="e" cm="1">
         <f t="array" aca="1" ref="M13" ca="1">_xll.one_touch_delta($C$2,I13,J13,$C$3,$C$6)</f>
-        <v>-8.4023712015289242E-3</v>
+        <v>#VALUE!</v>
       </c>
       <c r="X13" t="str">
-        <v>KXCANADAPM-45-C</v>
+        <v>KXCANADAPM-45-L</v>
       </c>
       <c r="Y13">
-        <v>2665960</v>
+        <v>3479711</v>
       </c>
       <c r="Z13">
-        <v>-10991</v>
+        <v>-7000</v>
       </c>
       <c r="AA13">
-        <v>727164</v>
+        <v>251557</v>
       </c>
       <c r="AB13">
-        <v>166704</v>
+        <v>-205253</v>
       </c>
       <c r="AC13">
-        <v>10764</v>
+        <v>4000</v>
       </c>
       <c r="AD13">
-        <v>15127</v>
+        <v>12724</v>
       </c>
       <c r="AE13" t="str">
-        <v>2025-04-09T18:08:13.280458Z</v>
+        <v>2025-04-10T12:09:54.480709Z</v>
       </c>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.25">
@@ -2172,16 +2151,16 @@
         <v>2026-01-01T04:59:00Z</v>
       </c>
       <c r="D14">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E14">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F14">
         <v>17</v>
       </c>
       <c r="G14">
-        <v>1584</v>
+        <v>1571</v>
       </c>
       <c r="H14" t="str">
         <v>less</v>
@@ -2192,54 +2171,54 @@
       <c r="J14">
         <v>1</v>
       </c>
-      <c r="K14" cm="1">
+      <c r="K14" t="e" cm="1">
         <f t="array" aca="1" ref="K14" ca="1">_xll.price_one_touch($C$2,I14,J14,$C$3,$C$6)</f>
-        <v>0.54104012670193768</v>
-      </c>
-      <c r="M14" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M14" t="e" cm="1">
         <f t="array" aca="1" ref="M14" ca="1">_xll.one_touch_delta($C$2,I14,J14,$C$3,$C$6)</f>
-        <v>-8.0356475393461579E-3</v>
+        <v>#VALUE!</v>
       </c>
       <c r="X14" t="str">
-        <v>KXNOBELPEACE-25-DJT</v>
+        <v>KXCANADAPM-45-C</v>
       </c>
       <c r="Y14">
-        <v>1032338</v>
+        <v>2665960</v>
       </c>
       <c r="Z14">
-        <v>-16</v>
+        <v>-10991</v>
       </c>
       <c r="AA14">
-        <v>1456</v>
+        <v>727164</v>
       </c>
       <c r="AB14">
-        <v>18518</v>
+        <v>166704</v>
       </c>
       <c r="AC14">
-        <v>0</v>
+        <v>10764</v>
       </c>
       <c r="AD14">
-        <v>0</v>
+        <v>15127</v>
       </c>
       <c r="AE14" t="str">
-        <v>2025-04-08T17:53:41.397741Z</v>
+        <v>2025-04-09T18:08:13.280458Z</v>
       </c>
     </row>
     <row r="15" spans="1:31" x14ac:dyDescent="0.25">
       <c r="X15" t="str">
-        <v>KXNOBELPEACE-25-JA</v>
+        <v>KXNOBELPEACE-25-DJT</v>
       </c>
       <c r="Y15">
-        <v>276</v>
+        <v>1032338</v>
       </c>
       <c r="Z15">
-        <v>-3</v>
+        <v>-16</v>
       </c>
       <c r="AA15">
-        <v>276</v>
+        <v>1456</v>
       </c>
       <c r="AB15">
-        <v>0</v>
+        <v>18518</v>
       </c>
       <c r="AC15">
         <v>0</v>
@@ -2248,33 +2227,33 @@
         <v>0</v>
       </c>
       <c r="AE15" t="str">
-        <v>2025-02-20T13:14:09.07897Z</v>
+        <v>2025-04-08T17:53:41.397741Z</v>
       </c>
     </row>
     <row r="16" spans="1:31" x14ac:dyDescent="0.25">
       <c r="X16" t="str">
-        <v>KXEXPAND-26</v>
+        <v>KXNOBELPEACE-25-JA</v>
       </c>
       <c r="Y16">
-        <v>820032</v>
+        <v>276</v>
       </c>
       <c r="Z16">
-        <v>-2528</v>
+        <v>-3</v>
       </c>
       <c r="AA16">
-        <v>242586</v>
+        <v>276</v>
       </c>
       <c r="AB16">
-        <v>9754</v>
+        <v>0</v>
       </c>
       <c r="AC16">
-        <v>3608</v>
+        <v>0</v>
       </c>
       <c r="AD16">
         <v>0</v>
       </c>
       <c r="AE16" t="str">
-        <v>2025-03-27T19:10:44.127655Z</v>
+        <v>2025-02-20T13:14:09.07897Z</v>
       </c>
     </row>
     <row r="17" spans="1:31" x14ac:dyDescent="0.25">
@@ -2285,28 +2264,28 @@
         <v>15</v>
       </c>
       <c r="X17" t="str">
-        <v>KXGOVTCUTS-25-750</v>
+        <v>KXEXPAND-26</v>
       </c>
       <c r="Y17">
-        <v>2953</v>
+        <v>820032</v>
       </c>
       <c r="Z17">
-        <v>-25</v>
+        <v>-2528</v>
       </c>
       <c r="AA17">
-        <v>2225</v>
+        <v>242586</v>
       </c>
       <c r="AB17">
-        <v>72</v>
+        <v>9754</v>
       </c>
       <c r="AC17">
+        <v>3608</v>
+      </c>
+      <c r="AD17">
         <v>0</v>
       </c>
-      <c r="AD17">
-        <v>6</v>
-      </c>
       <c r="AE17" t="str">
-        <v>2025-02-26T19:30:08.478399Z</v>
+        <v>2025-03-27T19:10:44.127655Z</v>
       </c>
     </row>
     <row r="18" spans="1:31" x14ac:dyDescent="0.25">
@@ -2357,28 +2336,28 @@
         <v>37</v>
       </c>
       <c r="X18" t="str">
-        <v>KXGOVTCUTS-25-1</v>
+        <v>KXGOVTCUTS-25-750</v>
       </c>
       <c r="Y18">
-        <v>572</v>
+        <v>2953</v>
       </c>
       <c r="Z18">
-        <v>-11</v>
+        <v>-25</v>
       </c>
       <c r="AA18">
-        <v>572</v>
+        <v>2225</v>
       </c>
       <c r="AB18">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="AC18">
         <v>0</v>
       </c>
       <c r="AD18">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE18" t="str">
-        <v>2025-03-08T19:48:48.60921Z</v>
+        <v>2025-02-26T19:30:08.478399Z</v>
       </c>
     </row>
     <row r="19" spans="1:31" x14ac:dyDescent="0.25">
@@ -2392,16 +2371,16 @@
         <v>2025-12-31T15:00:00Z</v>
       </c>
       <c r="D19">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E19">
+        <v>37</v>
+      </c>
+      <c r="F19">
         <v>36</v>
       </c>
-      <c r="F19">
-        <v>35</v>
-      </c>
       <c r="G19">
-        <v>2156</v>
+        <v>2368</v>
       </c>
       <c r="H19" t="str">
         <v>greater</v>
@@ -2409,37 +2388,37 @@
       <c r="I19">
         <v>124999.99</v>
       </c>
-      <c r="J19" s="5" cm="1">
+      <c r="J19" s="5" t="e" cm="1">
         <f t="array" aca="1" ref="J19" ca="1">_xll.generate_interpolation_function(I19,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.59243726673212294</v>
-      </c>
-      <c r="K19" s="6" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="K19" s="6" t="e" cm="1">
         <f t="array" aca="1" ref="K19" ca="1">_xll.price_one_touch($C$2,I19,J19,$C$3,$C$6)</f>
-        <v>0.30543192699043875</v>
+        <v>#VALUE!</v>
       </c>
       <c r="L19" cm="1">
         <f t="array" ref="L19">_xll.get_position(A19,_xlfn.ANCHORARRAY($X$2))</f>
-        <v>0</v>
-      </c>
-      <c r="M19" cm="1">
+        <v>1</v>
+      </c>
+      <c r="M19" t="e" cm="1">
         <f t="array" aca="1" ref="M19" ca="1">_xll.one_touch_delta($C$2,I19,J19,$C$3,$C$6)</f>
-        <v>1.1814977917919439E-2</v>
-      </c>
-      <c r="N19">
+        <v>#VALUE!</v>
+      </c>
+      <c r="N19" t="e">
         <f ca="1">L19*M19</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="X19" t="str">
-        <v>KXTIME-25-DT</v>
+        <v>KXGOVTCUTS-25-1</v>
       </c>
       <c r="Y19">
-        <v>1650</v>
+        <v>572</v>
       </c>
       <c r="Z19">
-        <v>-22</v>
+        <v>-11</v>
       </c>
       <c r="AA19">
-        <v>1650</v>
+        <v>572</v>
       </c>
       <c r="AB19">
         <v>0</v>
@@ -2451,7 +2430,7 @@
         <v>0</v>
       </c>
       <c r="AE19" t="str">
-        <v>2025-02-26T22:16:50.088515Z</v>
+        <v>2025-03-08T19:48:48.60921Z</v>
       </c>
     </row>
     <row r="20" spans="1:31" x14ac:dyDescent="0.25">
@@ -2482,37 +2461,37 @@
       <c r="I20">
         <v>149999.99</v>
       </c>
-      <c r="J20" s="5" cm="1">
+      <c r="J20" s="5" t="e" cm="1">
         <f t="array" aca="1" ref="J20" ca="1">_xll.generate_interpolation_function(I20,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.5690693897961665</v>
-      </c>
-      <c r="K20" s="6" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="K20" s="6" t="e" cm="1">
         <f t="array" aca="1" ref="K20" ca="1">_xll.price_one_touch($C$2,I20,J20,$C$3,$C$6)</f>
-        <v>0.12706061885307587</v>
+        <v>#VALUE!</v>
       </c>
       <c r="L20" cm="1">
         <f t="array" ref="L20">_xll.get_position(A20,_xlfn.ANCHORARRAY($X$2))</f>
         <v>1199</v>
       </c>
-      <c r="M20" cm="1">
+      <c r="M20" t="e" cm="1">
         <f t="array" aca="1" ref="M20" ca="1">_xll.one_touch_delta($C$2,I20,J20,$C$3,$C$6)</f>
-        <v>6.362289181448065E-3</v>
-      </c>
-      <c r="N20">
+        <v>#VALUE!</v>
+      </c>
+      <c r="N20" t="e">
         <f ca="1">L20*M20</f>
-        <v>7.6283847285562301</v>
+        <v>#VALUE!</v>
       </c>
       <c r="X20" t="str">
-        <v>KXTIME-25-GPT</v>
+        <v>KXTIME-25-DT</v>
       </c>
       <c r="Y20">
-        <v>95</v>
+        <v>1650</v>
       </c>
       <c r="Z20">
-        <v>-1</v>
+        <v>-22</v>
       </c>
       <c r="AA20">
-        <v>95</v>
+        <v>1650</v>
       </c>
       <c r="AB20">
         <v>0</v>
@@ -2521,10 +2500,10 @@
         <v>0</v>
       </c>
       <c r="AD20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE20" t="str">
-        <v>2025-02-26T03:44:14.890953Z</v>
+        <v>2025-02-26T22:16:50.088515Z</v>
       </c>
     </row>
     <row r="21" spans="1:31" x14ac:dyDescent="0.25">
@@ -2555,49 +2534,49 @@
       <c r="I21">
         <v>159999.99</v>
       </c>
-      <c r="J21" s="5" cm="1">
+      <c r="J21" s="5" t="e" cm="1">
         <f t="array" aca="1" ref="J21" ca="1">_xll.generate_interpolation_function(I21,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.56379718767571396</v>
-      </c>
-      <c r="K21" s="6" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="K21" s="6" t="e" cm="1">
         <f t="array" aca="1" ref="K21" ca="1">_xll.price_one_touch($C$2,I21,J21,$C$3,$C$6)</f>
-        <v>8.8506485427215481E-2</v>
+        <v>#VALUE!</v>
       </c>
       <c r="L21" cm="1">
         <f t="array" ref="L21">_xll.get_position(A21,_xlfn.ANCHORARRAY($X$2))</f>
         <v>500</v>
       </c>
-      <c r="M21" cm="1">
+      <c r="M21" t="e" cm="1">
         <f t="array" aca="1" ref="M21" ca="1">_xll.one_touch_delta($C$2,I21,J21,$C$3,$C$6)</f>
-        <v>4.8019426272631893E-3</v>
-      </c>
-      <c r="N21">
-        <f t="shared" ref="N21:N25" ca="1" si="0">L21*M21</f>
-        <v>2.4009713136315947</v>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N21" t="e">
+        <f ca="1">L21*M21</f>
+        <v>#VALUE!</v>
       </c>
       <c r="X21" t="str">
-        <v>KXDCEILEND-26</v>
+        <v>KXTIME-25-GPT</v>
       </c>
       <c r="Y21">
-        <v>23701</v>
+        <v>95</v>
       </c>
       <c r="Z21">
-        <v>-16</v>
+        <v>-1</v>
       </c>
       <c r="AA21">
-        <v>1280</v>
+        <v>95</v>
       </c>
       <c r="AB21">
-        <v>1179</v>
+        <v>0</v>
       </c>
       <c r="AC21">
         <v>0</v>
       </c>
       <c r="AD21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE21" t="str">
-        <v>2025-02-09T18:51:25.294953Z</v>
+        <v>2025-02-26T03:44:14.890953Z</v>
       </c>
     </row>
     <row r="22" spans="1:31" x14ac:dyDescent="0.25">
@@ -2620,7 +2599,7 @@
         <v>11</v>
       </c>
       <c r="G22">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H22" t="str">
         <v>greater</v>
@@ -2628,25 +2607,49 @@
       <c r="I22">
         <v>179999.99</v>
       </c>
-      <c r="J22" s="5" cm="1">
+      <c r="J22" s="5" t="e" cm="1">
         <f t="array" aca="1" ref="J22" ca="1">_xll.generate_interpolation_function(I22,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.56023840969868954</v>
-      </c>
-      <c r="K22" s="6" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="K22" s="6" t="e" cm="1">
         <f t="array" aca="1" ref="K22" ca="1">_xll.price_one_touch($C$2,I22,J22,$C$3,$C$6)</f>
-        <v>4.3830028856025355E-2</v>
+        <v>#VALUE!</v>
       </c>
       <c r="L22" cm="1">
         <f t="array" ref="L22">_xll.get_position(A22,_xlfn.ANCHORARRAY($X$2))</f>
         <v>543</v>
       </c>
-      <c r="M22" cm="1">
+      <c r="M22" t="e" cm="1">
         <f t="array" aca="1" ref="M22" ca="1">_xll.one_touch_delta($C$2,I22,J22,$C$3,$C$6)</f>
-        <v>2.690477789345308E-3</v>
-      </c>
-      <c r="N22">
+        <v>#VALUE!</v>
+      </c>
+      <c r="N22" t="e">
         <f ca="1">L22*M22</f>
-        <v>1.4609294396145023</v>
+        <v>#VALUE!</v>
+      </c>
+      <c r="X22" t="str">
+        <v>KXDCEILEND-26</v>
+      </c>
+      <c r="Y22">
+        <v>23701</v>
+      </c>
+      <c r="Z22">
+        <v>-16</v>
+      </c>
+      <c r="AA22">
+        <v>1280</v>
+      </c>
+      <c r="AB22">
+        <v>1179</v>
+      </c>
+      <c r="AC22">
+        <v>0</v>
+      </c>
+      <c r="AD22">
+        <v>0</v>
+      </c>
+      <c r="AE22" t="str">
+        <v>2025-02-09T18:51:25.294953Z</v>
       </c>
     </row>
     <row r="23" spans="1:31" x14ac:dyDescent="0.25">
@@ -2660,16 +2663,16 @@
         <v>2026-01-01T04:59:00Z</v>
       </c>
       <c r="D23">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E23">
         <v>13</v>
       </c>
       <c r="F23">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G23">
-        <v>1441</v>
+        <v>1835</v>
       </c>
       <c r="H23" t="str">
         <v>greater</v>
@@ -2677,25 +2680,25 @@
       <c r="I23">
         <v>199999.99</v>
       </c>
-      <c r="J23" s="5" cm="1">
+      <c r="J23" s="5" t="e" cm="1">
         <f t="array" aca="1" ref="J23" ca="1">_xll.generate_interpolation_function(I23,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.56599380007350542</v>
-      </c>
-      <c r="K23" s="6" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="K23" s="6" t="e" cm="1">
         <f t="array" aca="1" ref="K23" ca="1">_xll.price_one_touch($C$2,I23,J23,$C$3,$C$6)</f>
-        <v>2.3431290437650062E-2</v>
+        <v>#VALUE!</v>
       </c>
       <c r="L23" cm="1">
         <f t="array" ref="L23">_xll.get_position(A23,_xlfn.ANCHORARRAY($X$2))</f>
         <v>-2152</v>
       </c>
-      <c r="M23" cm="1">
+      <c r="M23" t="e" cm="1">
         <f t="array" aca="1" ref="M23" ca="1">_xll.one_touch_delta($C$2,I23,J23,$C$3,$C$6)</f>
-        <v>1.5537552347530507E-3</v>
-      </c>
-      <c r="N23">
+        <v>#VALUE!</v>
+      </c>
+      <c r="N23" t="e">
         <f ca="1">L23*M23</f>
-        <v>-3.343681265188565</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="24" spans="1:31" x14ac:dyDescent="0.25">
@@ -2709,16 +2712,16 @@
         <v>2026-01-01T04:59:00Z</v>
       </c>
       <c r="D24">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E24">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F24">
         <v>7</v>
       </c>
       <c r="G24">
-        <v>1825</v>
+        <v>2398</v>
       </c>
       <c r="H24" t="str">
         <v>greater</v>
@@ -2726,25 +2729,25 @@
       <c r="I24">
         <v>249999.99</v>
       </c>
-      <c r="J24" s="5" cm="1">
+      <c r="J24" s="5" t="e" cm="1">
         <f t="array" aca="1" ref="J24" ca="1">_xll.generate_interpolation_function(I24,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.62113176254984659</v>
-      </c>
-      <c r="K24" s="6" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="K24" s="6" t="e" cm="1">
         <f t="array" aca="1" ref="K24" ca="1">_xll.price_one_touch($C$2,I24,J24,$C$3,$C$6)</f>
-        <v>8.9871902556079401E-3</v>
+        <v>#VALUE!</v>
       </c>
       <c r="L24" cm="1">
         <f t="array" ref="L24">_xll.get_position(A24,_xlfn.ANCHORARRAY($X$2))</f>
         <v>-4539</v>
       </c>
-      <c r="M24" cm="1">
+      <c r="M24" t="e" cm="1">
         <f t="array" aca="1" ref="M24" ca="1">_xll.one_touch_delta($C$2,I24,J24,$C$3,$C$6)</f>
-        <v>6.0800365114045858E-4</v>
-      </c>
-      <c r="N24">
-        <f t="shared" ca="1" si="0"/>
-        <v>-2.7597285725265417</v>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N24" t="e">
+        <f ca="1">L24*M24</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="25" spans="1:31" x14ac:dyDescent="0.25">
@@ -2775,25 +2778,25 @@
       <c r="I25">
         <v>299999.99</v>
       </c>
-      <c r="J25" s="5" cm="1">
+      <c r="J25" s="5" t="e" cm="1">
         <f t="array" aca="1" ref="J25" ca="1">_xll.generate_interpolation_function(I25,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.73448327722519013</v>
-      </c>
-      <c r="K25" s="6" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="K25" s="6" t="e" cm="1">
         <f t="array" aca="1" ref="K25" ca="1">_xll.price_one_touch($C$2,I25,J25,$C$3,$C$6)</f>
-        <v>8.5659785514566652E-3</v>
+        <v>#VALUE!</v>
       </c>
       <c r="L25" cm="1">
         <f t="array" ref="L25">_xll.get_position(A25,_xlfn.ANCHORARRAY($X$2))</f>
         <v>-5780</v>
       </c>
-      <c r="M25" cm="1">
+      <c r="M25" t="e" cm="1">
         <f t="array" aca="1" ref="M25" ca="1">_xll.one_touch_delta($C$2,I25,J25,$C$3,$C$6)</f>
-        <v>4.9427492020814173E-4</v>
-      </c>
-      <c r="N25">
-        <f t="shared" ca="1" si="0"/>
-        <v>-2.8569090388030594</v>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N25" t="e">
+        <f ca="1">L25*M25</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="26" spans="1:31" x14ac:dyDescent="0.25">
@@ -2824,25 +2827,25 @@
       <c r="I26">
         <v>499999.99</v>
       </c>
-      <c r="J26" s="5" cm="1">
+      <c r="J26" s="5" t="e" cm="1">
         <f t="array" aca="1" ref="J26" ca="1">_xll.generate_interpolation_function(I26,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>1.7700248579165876</v>
-      </c>
-      <c r="K26" s="6" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="K26" s="6" t="e" cm="1">
         <f t="array" aca="1" ref="K26" ca="1">_xll.price_one_touch($C$2,I26,J26,$C$3,$C$6)</f>
-        <v>5.7397313250723614E-2</v>
+        <v>#VALUE!</v>
       </c>
       <c r="L26" cm="1">
         <f t="array" ref="L26">_xll.get_position(A26,_xlfn.ANCHORARRAY($X$2))</f>
         <v>-2052</v>
       </c>
-      <c r="M26" cm="1">
+      <c r="M26" t="e" cm="1">
         <f t="array" aca="1" ref="M26" ca="1">_xll.one_touch_delta($C$2,I26,J26,$C$3,$C$6)</f>
-        <v>1.1615606508868781E-3</v>
-      </c>
-      <c r="N26">
+        <v>#VALUE!</v>
+      </c>
+      <c r="N26" t="e">
         <f ca="1">L26*M26</f>
-        <v>-2.383522455619874</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="32" spans="1:31" x14ac:dyDescent="0.25">
@@ -2929,25 +2932,25 @@
       <c r="C36" t="s">
         <v>31</v>
       </c>
-      <c r="D36" cm="1">
+      <c r="D36" t="e" cm="1">
         <f t="array" aca="1" ref="D36" ca="1">_xll.find_strike(D33,D35,$C$6,$C$2,$C$3,0,D34)</f>
-        <v>35114.280341540543</v>
-      </c>
-      <c r="E36" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E36" t="e" cm="1">
         <f t="array" aca="1" ref="E36" ca="1">_xll.find_strike(E33,E35,$C$6,$C$2,$C$3,0,E34)</f>
-        <v>71098.823521647369</v>
-      </c>
-      <c r="F36" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F36" t="e" cm="1">
         <f t="array" aca="1" ref="F36" ca="1">_xll.find_strike(F33,F35,$C$6,$C$2,$C$3,0,F34)</f>
-        <v>98737.330303366325</v>
-      </c>
-      <c r="G36" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G36" t="e" cm="1">
         <f t="array" aca="1" ref="G36" ca="1">_xll.find_strike(G33,G35,$C$6,$C$2,$C$3,0,G34)</f>
-        <v>149456.10652824733</v>
-      </c>
-      <c r="H36" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="H36" t="e" cm="1">
         <f t="array" aca="1" ref="H36" ca="1">_xll.find_strike(H33,H35,$C$6,$C$2,$C$3,0,H34)</f>
-        <v>308288.55334553076</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.25">
@@ -2960,9 +2963,9 @@
         <f>50000</f>
         <v>50000</v>
       </c>
-      <c r="C42" cm="1">
+      <c r="C42" t="e" cm="1">
         <f t="array" aca="1" ref="C42" ca="1">_xll.generate_interpolation_function(B42,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.74986119611660285</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.25">
@@ -2970,239 +2973,239 @@
         <f>B42+10000</f>
         <v>60000</v>
       </c>
-      <c r="C43" cm="1">
+      <c r="C43" t="e" cm="1">
         <f t="array" aca="1" ref="C43" ca="1">_xll.generate_interpolation_function(B43,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.7213035754450916</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B44">
-        <f t="shared" ref="B44:B66" si="1">B43+10000</f>
+        <f t="shared" ref="B44:B66" si="0">B43+10000</f>
         <v>70000</v>
       </c>
-      <c r="C44" cm="1">
+      <c r="C44" t="e" cm="1">
         <f t="array" aca="1" ref="C44" ca="1">_xll.generate_interpolation_function(B44,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.69507449686154033</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B45">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>80000</v>
       </c>
-      <c r="C45" cm="1">
+      <c r="C45" t="e" cm="1">
         <f t="array" aca="1" ref="C45" ca="1">_xll.generate_interpolation_function(B45,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.67117396036594934</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>90000</v>
       </c>
-      <c r="C46" cm="1">
+      <c r="C46" t="e" cm="1">
         <f t="array" aca="1" ref="C46" ca="1">_xll.generate_interpolation_function(B46,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.64960196595831832</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B47">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>100000</v>
       </c>
-      <c r="C47" cm="1">
+      <c r="C47" t="e" cm="1">
         <f t="array" aca="1" ref="C47" ca="1">_xll.generate_interpolation_function(B47,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.63035851363864748</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B48">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>110000</v>
       </c>
-      <c r="C48" cm="1">
+      <c r="C48" t="e" cm="1">
         <f t="array" aca="1" ref="C48" ca="1">_xll.generate_interpolation_function(B48,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.61344360340693671</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B49">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>120000</v>
       </c>
-      <c r="C49" cm="1">
+      <c r="C49" t="e" cm="1">
         <f t="array" aca="1" ref="C49" ca="1">_xll.generate_interpolation_function(B49,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.59885723526318602</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="50" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B50">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>130000</v>
       </c>
-      <c r="C50" cm="1">
+      <c r="C50" t="e" cm="1">
         <f t="array" aca="1" ref="C50" ca="1">_xll.generate_interpolation_function(B50,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.58659940920739539</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="51" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B51">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>140000</v>
       </c>
-      <c r="C51" cm="1">
+      <c r="C51" t="e" cm="1">
         <f t="array" aca="1" ref="C51" ca="1">_xll.generate_interpolation_function(B51,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.57667012523956485</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B52">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>150000</v>
       </c>
-      <c r="C52" cm="1">
+      <c r="C52" t="e" cm="1">
         <f t="array" aca="1" ref="C52" ca="1">_xll.generate_interpolation_function(B52,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.56906938335969448</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="53" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B53">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>160000</v>
       </c>
-      <c r="C53" cm="1">
+      <c r="C53" t="e" cm="1">
         <f t="array" aca="1" ref="C53" ca="1">_xll.generate_interpolation_function(B53,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.56379718356778419</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="54" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B54">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>170000</v>
       </c>
-      <c r="C54" cm="1">
+      <c r="C54" t="e" cm="1">
         <f t="array" aca="1" ref="C54" ca="1">_xll.generate_interpolation_function(B54,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.56085352586383386</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B55">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>180000</v>
       </c>
-      <c r="C55" cm="1">
+      <c r="C55" t="e" cm="1">
         <f t="array" aca="1" ref="C55" ca="1">_xll.generate_interpolation_function(B55,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.56023841024784382</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="56" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B56">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>190000</v>
       </c>
-      <c r="C56" cm="1">
+      <c r="C56" t="e" cm="1">
         <f t="array" aca="1" ref="C56" ca="1">_xll.generate_interpolation_function(B56,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.56195183671981375</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B57">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>200000</v>
       </c>
-      <c r="C57" cm="1">
+      <c r="C57" t="e" cm="1">
         <f t="array" aca="1" ref="C57" ca="1">_xll.generate_interpolation_function(B57,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.56599380527974386</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="58" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B58">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>210000</v>
       </c>
-      <c r="C58" cm="1">
+      <c r="C58" t="e" cm="1">
         <f t="array" aca="1" ref="C58" ca="1">_xll.generate_interpolation_function(B58,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.57236431592763393</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="59" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B59">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>220000</v>
       </c>
-      <c r="C59" cm="1">
+      <c r="C59" t="e" cm="1">
         <f t="array" aca="1" ref="C59" ca="1">_xll.generate_interpolation_function(B59,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.58106336866348418</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B60">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>230000</v>
       </c>
-      <c r="C60" cm="1">
+      <c r="C60" t="e" cm="1">
         <f t="array" aca="1" ref="C60" ca="1">_xll.generate_interpolation_function(B60,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.59209096348729451</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="61" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B61">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>240000</v>
       </c>
-      <c r="C61" cm="1">
+      <c r="C61" t="e" cm="1">
         <f t="array" aca="1" ref="C61" ca="1">_xll.generate_interpolation_function(B61,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.60544710039906491</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="62" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B62">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>250000</v>
       </c>
-      <c r="C62" cm="1">
+      <c r="C62" t="e" cm="1">
         <f t="array" aca="1" ref="C62" ca="1">_xll.generate_interpolation_function(B62,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.62113177939879549</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B63">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>260000</v>
       </c>
-      <c r="C63" cm="1">
+      <c r="C63" t="e" cm="1">
         <f t="array" aca="1" ref="C63" ca="1">_xll.generate_interpolation_function(B63,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.63914500048648615</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="64" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B64">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>270000</v>
       </c>
-      <c r="C64" cm="1">
+      <c r="C64" t="e" cm="1">
         <f t="array" aca="1" ref="C64" ca="1">_xll.generate_interpolation_function(B64,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.65948676366213677</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="65" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B65">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>280000</v>
       </c>
-      <c r="C65" cm="1">
+      <c r="C65" t="e" cm="1">
         <f t="array" aca="1" ref="C65" ca="1">_xll.generate_interpolation_function(B65,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.68215706892574757</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B66">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>290000</v>
       </c>
-      <c r="C66" cm="1">
+      <c r="C66" t="e" cm="1">
         <f t="array" aca="1" ref="C66" ca="1">_xll.generate_interpolation_function(B66,$D$36:$H$36,$D$35:$H$35)</f>
-        <v>0.70715591627731855</v>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
@@ -3232,9 +3235,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="str" cm="1">
-        <f t="array" ref="A1">_xll.get_events("Crypto")</f>
-        <v>##FileNotFoundError: [Errno 2] No such file or directory: 'mkt_key_2.txt'</v>
+      <c r="A1" t="e" cm="1">
+        <f t="array" aca="1" ref="A1" ca="1">_xll.get_events("Crypto")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
@@ -3269,57 +3272,57 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B2">
-        <f>C2-500</f>
-        <v>-850.27001953125</v>
-      </c>
-      <c r="C2">
-        <f>D2-500</f>
-        <v>-350.27001953125</v>
-      </c>
-      <c r="D2">
-        <f>E2-500</f>
-        <v>149.72998046875</v>
-      </c>
-      <c r="E2">
-        <f>F2-500</f>
-        <v>649.72998046875</v>
-      </c>
-      <c r="F2">
-        <f>G2-500</f>
-        <v>1149.72998046875</v>
-      </c>
-      <c r="G2">
-        <f>Sheet1!B2</f>
-        <v>1649.72998046875</v>
-      </c>
-      <c r="H2">
-        <f t="shared" ref="H2:N2" si="0">G2+500</f>
-        <v>2149.72998046875</v>
-      </c>
-      <c r="I2">
-        <f t="shared" si="0"/>
-        <v>2649.72998046875</v>
-      </c>
-      <c r="J2">
-        <f t="shared" si="0"/>
-        <v>3149.72998046875</v>
-      </c>
-      <c r="K2">
-        <f t="shared" si="0"/>
-        <v>3649.72998046875</v>
-      </c>
-      <c r="L2">
-        <f t="shared" si="0"/>
-        <v>4149.72998046875</v>
-      </c>
-      <c r="M2">
-        <f t="shared" si="0"/>
-        <v>4649.72998046875</v>
-      </c>
-      <c r="N2">
-        <f t="shared" si="0"/>
-        <v>5149.72998046875</v>
+      <c r="B2" t="e">
+        <f ca="1">C2-500</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C2" t="e">
+        <f ca="1">D2-500</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D2" t="e">
+        <f ca="1">E2-500</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E2" t="e">
+        <f ca="1">F2-500</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="F2" t="e">
+        <f ca="1">G2-500</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="G2" t="e">
+        <f ca="1">Sheet1!B2</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="H2" t="e">
+        <f t="shared" ref="H2:N2" ca="1" si="0">G2+500</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I2" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="J2" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K2" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L2" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M2" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N2" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">

</xml_diff>